<commit_message>
✅ test(api): update help route and reporter fixture
</commit_message>
<xml_diff>
--- a/tests/fixtures/resources/results/profile_report.xlsx
+++ b/tests/fixtures/resources/results/profile_report.xlsx
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="profile_report" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
@@ -130,6 +130,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -625,9 +628,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% — акцент1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1033,9 +1037,7 @@
       <c r="I2">
         <v>150</v>
       </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
+      <c r="M2" s="2"/>
       <c r="O2">
         <v>1</v>
       </c>
@@ -1043,7 +1045,7 @@
         <v>0</v>
       </c>
       <c r="Q2">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -1074,9 +1076,7 @@
       <c r="I3">
         <v>150</v>
       </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
+      <c r="M3" s="2"/>
       <c r="O3">
         <v>1</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>0</v>
       </c>
       <c r="Q3">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -1115,9 +1115,7 @@
       <c r="I4">
         <v>70</v>
       </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
+      <c r="M4" s="2"/>
       <c r="O4">
         <v>1</v>
       </c>
@@ -1125,7 +1123,7 @@
         <v>0</v>
       </c>
       <c r="Q4">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -1165,7 +1163,7 @@
       <c r="L5" t="s">
         <v>25</v>
       </c>
-      <c r="M5">
+      <c r="M5" s="2">
         <v>5</v>
       </c>
       <c r="O5">
@@ -1215,7 +1213,7 @@
       <c r="L6" t="s">
         <v>26</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="2">
         <v>15</v>
       </c>
       <c r="O6">
@@ -1265,7 +1263,7 @@
       <c r="L7" t="s">
         <v>27</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="2">
         <v>10</v>
       </c>
       <c r="O7">
@@ -1315,7 +1313,7 @@
       <c r="L8" t="s">
         <v>28</v>
       </c>
-      <c r="M8">
+      <c r="M8" s="2">
         <v>20</v>
       </c>
       <c r="O8">
@@ -1365,7 +1363,7 @@
       <c r="L9" t="s">
         <v>29</v>
       </c>
-      <c r="M9">
+      <c r="M9" s="2">
         <v>30</v>
       </c>
       <c r="O9">
@@ -1415,7 +1413,7 @@
       <c r="L10" t="s">
         <v>30</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="2">
         <v>10</v>
       </c>
       <c r="O10">
@@ -1465,7 +1463,7 @@
       <c r="L11" t="s">
         <v>31</v>
       </c>
-      <c r="M11">
+      <c r="M11" s="2">
         <v>10</v>
       </c>
       <c r="O11">
@@ -1515,7 +1513,7 @@
       <c r="L12" t="s">
         <v>25</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="2">
         <v>5</v>
       </c>
       <c r="O12">
@@ -1565,7 +1563,7 @@
       <c r="L13" t="s">
         <v>26</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="2">
         <v>15</v>
       </c>
       <c r="O13">
@@ -1615,7 +1613,7 @@
       <c r="L14" t="s">
         <v>27</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="2">
         <v>10</v>
       </c>
       <c r="O14">
@@ -1665,7 +1663,7 @@
       <c r="L15" t="s">
         <v>28</v>
       </c>
-      <c r="M15">
+      <c r="M15" s="2">
         <v>20</v>
       </c>
       <c r="O15">
@@ -1715,7 +1713,7 @@
       <c r="L16" t="s">
         <v>29</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="2">
         <v>30</v>
       </c>
       <c r="O16">
@@ -1765,7 +1763,7 @@
       <c r="L17" t="s">
         <v>30</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="2">
         <v>10</v>
       </c>
       <c r="O17">
@@ -1815,7 +1813,7 @@
       <c r="L18" t="s">
         <v>31</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="2">
         <v>10</v>
       </c>
       <c r="O18">
@@ -1856,14 +1854,12 @@
       <c r="I19">
         <v>0</v>
       </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
+      <c r="M19" s="2"/>
       <c r="O19">
         <v>1</v>
       </c>
       <c r="P19">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="Q19">
         <v>0</v>
@@ -1897,14 +1893,12 @@
       <c r="I20">
         <v>0</v>
       </c>
-      <c r="M20">
-        <v>0</v>
-      </c>
+      <c r="M20" s="2"/>
       <c r="O20">
         <v>1</v>
       </c>
       <c r="P20">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="Q20">
         <v>0</v>
@@ -1938,14 +1932,12 @@
       <c r="I21">
         <v>0</v>
       </c>
-      <c r="M21">
-        <v>0</v>
-      </c>
+      <c r="M21" s="2"/>
       <c r="O21">
         <v>1</v>
       </c>
       <c r="P21">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="Q21">
         <v>0</v>
@@ -1979,14 +1971,12 @@
       <c r="I22">
         <v>0</v>
       </c>
-      <c r="M22">
-        <v>0</v>
-      </c>
+      <c r="M22" s="2"/>
       <c r="O22">
         <v>1</v>
       </c>
       <c r="P22">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="Q22">
         <v>0</v>

</xml_diff>